<commit_message>
chore: bump version to 0.4.16
</commit_message>
<xml_diff>
--- a/data/test/order-day-addresses.xlsx
+++ b/data/test/order-day-addresses.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -459,9 +459,49 @@
         <v>2026-05-09T04:29:01.442Z</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>test-sub-0901000009-2026-W22-3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>test-sub-0901000009</v>
+      </c>
+      <c r="C4" t="str">
+        <v>2026-W22</v>
+      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="E4" t="str">
+        <v>test-addr-0901000009-1</v>
+      </c>
+      <c r="F4" t="str">
+        <v>2026-05-27T05:46:20.212Z</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>test-sub-0901000013-2026-W22-5</v>
+      </c>
+      <c r="B5" t="str">
+        <v>test-sub-0901000013</v>
+      </c>
+      <c r="C5" t="str">
+        <v>2026-W22</v>
+      </c>
+      <c r="D5">
+        <v>5</v>
+      </c>
+      <c r="E5" t="str">
+        <v>test-addr-0901000013-0</v>
+      </c>
+      <c r="F5" t="str">
+        <v>2026-05-27T05:47:54.559Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>